<commit_message>
Reconcile domain overview and batch counts to 896 strictly for 4 operational batches
</commit_message>
<xml_diff>
--- a/public/reports/Cards_Summary_Pending_Audit.xlsx
+++ b/public/reports/Cards_Summary_Pending_Audit.xlsx
@@ -398,7 +398,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:B53"/>
+  <dimension ref="A1:B44"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -415,7 +415,7 @@
         <v>Total no of Complaints</v>
       </c>
       <c r="B3">
-        <v>904</v>
+        <v>896</v>
       </c>
     </row>
     <row r="4">
@@ -431,7 +431,7 @@
         <v>Total no of Payment Pending Cases</v>
       </c>
       <c r="B5">
-        <v>274</v>
+        <v>272</v>
       </c>
     </row>
     <row r="6">
@@ -439,7 +439,7 @@
         <v>Total no of PO Pending Cases</v>
       </c>
       <c r="B6">
-        <v>307</v>
+        <v>304</v>
       </c>
     </row>
     <row r="7">
@@ -447,7 +447,7 @@
         <v>Total no of Inprocess Cases</v>
       </c>
       <c r="B7">
-        <v>118</v>
+        <v>113</v>
       </c>
     </row>
     <row r="8">
@@ -455,7 +455,7 @@
         <v>Total no of Cancel Cases</v>
       </c>
       <c r="B8">
-        <v>136</v>
+        <v>138</v>
       </c>
     </row>
     <row r="10">
@@ -497,7 +497,7 @@
         <v>Total no of PO Pending Cases</v>
       </c>
       <c r="B15">
-        <v>118</v>
+        <v>117</v>
       </c>
     </row>
     <row r="16">
@@ -505,7 +505,7 @@
         <v>Total no of Inprocess Cases</v>
       </c>
       <c r="B16">
-        <v>23</v>
+        <v>22</v>
       </c>
     </row>
     <row r="17">
@@ -513,7 +513,7 @@
         <v>Total no of Cancel Cases</v>
       </c>
       <c r="B17">
-        <v>46</v>
+        <v>48</v>
       </c>
     </row>
     <row r="19">
@@ -690,67 +690,9 @@
         <v>13</v>
       </c>
     </row>
-    <row r="46">
-      <c r="A46" t="str">
-        <v>Domain Overview</v>
-      </c>
-    </row>
-    <row r="47">
-      <c r="A47" t="str">
-        <v>Unassigned</v>
-      </c>
-    </row>
-    <row r="48">
-      <c r="A48" t="str">
-        <v>Total no of Complaints</v>
-      </c>
-      <c r="B48">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="49">
-      <c r="A49" t="str">
-        <v>Total no of Payment Received Cases</v>
-      </c>
-      <c r="B49">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="50">
-      <c r="A50" t="str">
-        <v>Total no of Payment Pending Cases</v>
-      </c>
-      <c r="B50">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="51">
-      <c r="A51" t="str">
-        <v>Total no of PO Pending Cases</v>
-      </c>
-      <c r="B51">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="52">
-      <c r="A52" t="str">
-        <v>Total no of Inprocess Cases</v>
-      </c>
-      <c r="B52">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="53">
-      <c r="A53" t="str">
-        <v>Total no of Cancel Cases</v>
-      </c>
-      <c r="B53">
-        <v>0</v>
-      </c>
-    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:B53"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:B44"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -803,7 +745,7 @@
         <v>Total no of PO Pending Cases</v>
       </c>
       <c r="B8">
-        <v>31</v>
+        <v>30</v>
       </c>
     </row>
     <row r="9">
@@ -819,7 +761,7 @@
         <v>Total no of Cancel Cases</v>
       </c>
       <c r="B10">
-        <v>7</v>
+        <v>8</v>
       </c>
     </row>
     <row r="12">
@@ -1011,7 +953,7 @@
         <v>Total no of Complaints</v>
       </c>
       <c r="B41">
-        <v>63</v>
+        <v>62</v>
       </c>
     </row>
     <row r="42">
@@ -1027,7 +969,7 @@
         <v>Total no of Payment Pending Cases</v>
       </c>
       <c r="B43">
-        <v>22</v>
+        <v>21</v>
       </c>
     </row>
     <row r="44">
@@ -1069,7 +1011,7 @@
         <v>Total no of Complaints</v>
       </c>
       <c r="B50">
-        <v>147</v>
+        <v>145</v>
       </c>
     </row>
     <row r="51">
@@ -1093,7 +1035,7 @@
         <v>Total no of PO Pending Cases</v>
       </c>
       <c r="B53">
-        <v>35</v>
+        <v>34</v>
       </c>
     </row>
     <row r="54">
@@ -1101,7 +1043,7 @@
         <v>Total no of Inprocess Cases</v>
       </c>
       <c r="B54">
-        <v>23</v>
+        <v>22</v>
       </c>
     </row>
     <row r="55">
@@ -1127,7 +1069,7 @@
         <v>Total no of Complaints</v>
       </c>
       <c r="B59">
-        <v>193</v>
+        <v>189</v>
       </c>
     </row>
     <row r="60">
@@ -1143,7 +1085,7 @@
         <v>Total no of Payment Pending Cases</v>
       </c>
       <c r="B61">
-        <v>55</v>
+        <v>54</v>
       </c>
     </row>
     <row r="62">
@@ -1151,7 +1093,7 @@
         <v>Total no of PO Pending Cases</v>
       </c>
       <c r="B62">
-        <v>47</v>
+        <v>46</v>
       </c>
     </row>
     <row r="63">
@@ -1159,7 +1101,7 @@
         <v>Total no of Inprocess Cases</v>
       </c>
       <c r="B63">
-        <v>28</v>
+        <v>26</v>
       </c>
     </row>
     <row r="64">
@@ -1185,7 +1127,7 @@
         <v>Total no of Complaints</v>
       </c>
       <c r="B68">
-        <v>63</v>
+        <v>62</v>
       </c>
     </row>
     <row r="69">
@@ -1217,7 +1159,7 @@
         <v>Total no of Inprocess Cases</v>
       </c>
       <c r="B72">
-        <v>6</v>
+        <v>4</v>
       </c>
     </row>
     <row r="73">
@@ -1225,7 +1167,7 @@
         <v>Total no of Cancel Cases</v>
       </c>
       <c r="B73">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="75">

</xml_diff>